<commit_message>
docs: describe project components by pipeline role
</commit_message>
<xml_diff>
--- a/docs/data_sources.xlsx
+++ b/docs/data_sources.xlsx
@@ -686,7 +686,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Người 1</t>
+          <t>Listing Pipeline</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -828,7 +828,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Người 2</t>
+          <t>Location Mapping</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Người 2</t>
+          <t>Location Mapping</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">

</xml_diff>